<commit_message>
Finalize reviewed recipes and update tracker
</commit_message>
<xml_diff>
--- a/data/recepten/review-overzicht.xlsx
+++ b/data/recepten/review-overzicht.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Receptenoverzicht" sheetId="1" r:id="Rf742baa54784481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Werkwijze" sheetId="2" r:id="Ra5d1ba5a3f29423b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Receptenoverzicht" sheetId="1" r:id="Rb93ed3bb7a9a4a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Werkwijze" sheetId="2" r:id="R255dacaed297481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statusoverzicht" sheetId="3" r:id="R3594385f7a2848be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +27,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -38,6 +39,26 @@
         <x:fgColor rgb="FF604431"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF204A43"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCFCE7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -46,7 +67,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -68,6 +89,21 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -290,59 +326,59 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="35" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="56" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="34" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="29" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="35" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="12" t="str">
         <x:v>Sleutel</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="12" t="str">
         <x:v>Recept</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>Keuken/regio</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>Reviewstatus</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>Beschrijving</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>Ingrediënten</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>Bereiding</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>Bron</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="12" t="str">
         <x:v>Website/JSON</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="J1" s="12" t="str">
         <x:v>Volgende actie</x:v>
       </x:c>
-      <x:c r="K1" s="4" t="str">
+      <x:c r="K1" s="12" t="str">
         <x:v>Bestandspad</x:v>
       </x:c>
-      <x:c r="L1" s="4" t="str">
+      <x:c r="L1" s="12" t="str">
         <x:v>Herkomst</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="45" customHeight="1">
+    <x:row r="2" ht="55" customHeight="1">
       <x:c r="A2" s="8" t="str">
         <x:v>rendang</x:v>
       </x:c>
@@ -352,7 +388,7 @@
       <x:c r="C2" s="8" t="str">
         <x:v>Maleis-Indonesisch</x:v>
       </x:c>
-      <x:c r="D2" s="8" t="str">
+      <x:c r="D2" s="13" t="str">
         <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E2" s="8" t="str">
@@ -368,10 +404,10 @@
         <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I2" s="8" t="str">
-        <x:v>Nog verwerken</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J2" s="8" t="str">
-        <x:v>Persoonlijke definitieve tekst/hoeveelheden/stappen overzetten naar JSON; daarna index bijwerken</x:v>
+        <x:v>Controleer definitieve JSON, bouw index en commit zo nodig.</x:v>
       </x:c>
       <x:c r="K2" s="8" t="str">
         <x:v>data/recepten/rendang.json</x:v>
@@ -380,7 +416,7 @@
         <x:v>Hoofdchat</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="45" customHeight="1">
+    <x:row r="3" ht="55" customHeight="1">
       <x:c r="A3" s="8" t="str">
         <x:v>sate-ayam</x:v>
       </x:c>
@@ -390,26 +426,26 @@
       <x:c r="C3" s="8" t="str">
         <x:v>Maleis-Indonesisch</x:v>
       </x:c>
-      <x:c r="D3" s="8" t="str">
-        <x:v>In review</x:v>
+      <x:c r="D3" s="13" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E3" s="8" t="str">
         <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F3" s="8" t="str">
-        <x:v>In review</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="G3" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="H3" s="8" t="str">
         <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I3" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J3" s="8" t="str">
-        <x:v>Ingrediëntenlijst controleren (vier personen, marinades); daarna stappen reviewen</x:v>
+        <x:v>Controleer data/recepten/sate-ayam.json en afbeelding SateAjamAI.png.</x:v>
       </x:c>
       <x:c r="K3" s="8" t="str">
         <x:v>data/recepten/sate-ayam.json</x:v>
@@ -418,9 +454,9 @@
         <x:v>Hoofdchat</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="45" customHeight="1">
+    <x:row r="4" ht="55" customHeight="1">
       <x:c r="A4" s="8" t="str">
-        <x:v>nasi-goreng-bacon</x:v>
+        <x:v>nasiGoreng</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
         <x:v>Nasi goreng bacon</x:v>
@@ -428,37 +464,37 @@
       <x:c r="C4" s="8" t="str">
         <x:v>Maleis-Indonesisch</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="str">
-        <x:v>Klaar voor review</x:v>
+      <x:c r="D4" s="13" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E4" s="8" t="str">
         <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F4" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="G4" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="H4" s="8" t="str">
         <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I4" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J4" s="8" t="str">
-        <x:v>Hoeveelheden en bereiding reviewen; rijst en spekvolgorde controleren</x:v>
+        <x:v>Controleer bestaande sleutel nasiGoreng en receptpagina na indexbouw.</x:v>
       </x:c>
       <x:c r="K4" s="8" t="str">
-        <x:v>data/recepten/nasi-goreng-bacon.json</x:v>
+        <x:v>data/recepten/nasiGoreng.json</x:v>
       </x:c>
       <x:c r="L4" s="8" t="str">
         <x:v>Hoofdchat</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="45" customHeight="1">
+    <x:row r="5" ht="55" customHeight="1">
       <x:c r="A5" s="8" t="str">
-        <x:v>gado-gado</x:v>
+        <x:v>gadoGado</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
         <x:v>Gado gado</x:v>
@@ -466,111 +502,111 @@
       <x:c r="C5" s="8" t="str">
         <x:v>Maleis-Indonesisch</x:v>
       </x:c>
-      <x:c r="D5" s="8" t="str">
-        <x:v>Klaar voor review</x:v>
+      <x:c r="D5" s="13" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E5" s="8" t="str">
         <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F5" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="G5" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="H5" s="8" t="str">
         <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I5" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J5" s="8" t="str">
-        <x:v>Ingrediënten en groenten afstemmen; vloeibare satésaus uitwerken</x:v>
+        <x:v>Controleer receptbestand en afbeelding zonder taugé.</x:v>
       </x:c>
       <x:c r="K5" s="8" t="str">
-        <x:v>data/recepten/gado-gado.json</x:v>
+        <x:v>data/recepten/gadoGado.json</x:v>
       </x:c>
       <x:c r="L5" s="8" t="str">
         <x:v>Hoofdchat</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="45" customHeight="1">
+    <x:row r="6" ht="55" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>peking-eend</x:v>
+        <x:v>pekingEend</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>Chinese geroosterde eend (Peking-stijl)</x:v>
+        <x:v>Peking-eend met Chinese pannenkoekjes</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Chinees</x:v>
       </x:c>
-      <x:c r="D6" s="8" t="str">
-        <x:v>Concept – historische basis</x:v>
+      <x:c r="D6" s="13" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F6" s="8" t="str">
-        <x:v>Historische basis</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="G6" s="8" t="str">
-        <x:v>Nog veilig uitwerken</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="H6" s="8" t="str">
         <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I6" s="8" t="str">
-        <x:v>Concept</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J6" s="8" t="str">
-        <x:v>Moderne, veilige thuisbereiding uitwerken; zout en gaartijd verifiëren</x:v>
+        <x:v>Controleer Peking-eend JSON, historisch weetje en script/CSS-weergave.</x:v>
       </x:c>
       <x:c r="K6" s="8" t="str">
-        <x:v>Nog toe te wijzen</x:v>
+        <x:v>data/recepten/pekingEend.json</x:v>
       </x:c>
       <x:c r="L6" s="8" t="str">
         <x:v>Hoofdchat</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="45" customHeight="1">
+    <x:row r="7" ht="55" customHeight="1">
       <x:c r="A7" s="8" t="str">
-        <x:v>coq-au-vin</x:v>
+        <x:v>coqAuVin</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>Coq au vin (Mary Berry)</x:v>
+        <x:v>Coq au vin</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Frans</x:v>
       </x:c>
-      <x:c r="D7" s="8" t="str">
-        <x:v>Concept – in review</x:v>
+      <x:c r="D7" s="13" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E7" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F7" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="G7" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="H7" s="8" t="str">
         <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I7" s="8" t="str">
-        <x:v>Niet gepubliceerd</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
-        <x:v>Champignons (meestoven of apart bakken) en tijm beoordelen</x:v>
+        <x:v>Controleer juiste plaatsing van de definitieve JSON.</x:v>
       </x:c>
       <x:c r="K7" s="8" t="str">
-        <x:v>Nog toe te wijzen</x:v>
+        <x:v>data/recepten/coqAuVin.json</x:v>
       </x:c>
       <x:c r="L7" s="8" t="str">
-        <x:v>Telefoonchat; eerdere context</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="45" customHeight="1">
+        <x:v>Hoofdchat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="55" customHeight="1">
       <x:c r="A8" s="8" t="str">
         <x:v>hutspot-1601</x:v>
       </x:c>
@@ -580,73 +616,73 @@
       <x:c r="C8" s="8" t="str">
         <x:v>Nederlands historisch</x:v>
       </x:c>
-      <x:c r="D8" s="8" t="str">
-        <x:v>Concept – in review</x:v>
+      <x:c r="D8" s="14" t="str">
+        <x:v>Geïntegreerd als weetje</x:v>
       </x:c>
       <x:c r="E8" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F8" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Niet van toepassing</x:v>
       </x:c>
       <x:c r="G8" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Niet van toepassing</x:v>
       </x:c>
       <x:c r="H8" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I8" s="8" t="str">
-        <x:v>Niet gepubliceerd</x:v>
+        <x:v>Geen apart recept</x:v>
       </x:c>
       <x:c r="J8" s="8" t="str">
-        <x:v>Historische rundvleesstoofpot zonder aardappelen/wortelen; recept en bron controleren</x:v>
+        <x:v>Historisch weetje opgenomen bij stamppot; eventueel oude concepten opruimen.</x:v>
       </x:c>
       <x:c r="K8" s="8" t="str">
-        <x:v>Nog toe te wijzen</x:v>
+        <x:v>Geen afzonderlijk recept</x:v>
       </x:c>
       <x:c r="L8" s="8" t="str">
-        <x:v>Telefoonchat; eerdere context</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="45" customHeight="1">
+        <x:v>Hoofdchat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="55" customHeight="1">
       <x:c r="A9" s="8" t="str">
-        <x:v>hutspot-modern</x:v>
+        <x:v>stamppot</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>Moderne hutspot</x:v>
+        <x:v>Hutspot met rookworst</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>Nederlands</x:v>
-      </x:c>
-      <x:c r="D9" s="8" t="str">
-        <x:v>Concept – in review</x:v>
+        <x:v>Nederlands / Germaans</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
       </x:c>
       <x:c r="E9" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="F9" s="8" t="str">
-        <x:v>Voorlopig</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="G9" s="8" t="str">
-        <x:v>Voorlopig</x:v>
+        <x:v>Goedgekeurd</x:v>
       </x:c>
       <x:c r="H9" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Bekend</x:v>
       </x:c>
       <x:c r="I9" s="8" t="str">
-        <x:v>Niet gepubliceerd</x:v>
+        <x:v>Publicatie controleren</x:v>
       </x:c>
       <x:c r="J9" s="8" t="str">
-        <x:v>Aardappel, winterpeen, ui, rookworst; hoeveelheden en bereidingswijze afronden</x:v>
+        <x:v>Vervang stamppot.json, controleer historisch weetje; vervang StamppotAI.png met goedgekeurde afbeelding; verwijder oude hutspot-concepten.</x:v>
       </x:c>
       <x:c r="K9" s="8" t="str">
-        <x:v>Nog toe te wijzen</x:v>
+        <x:v>data/recepten/stamppot.json</x:v>
       </x:c>
       <x:c r="L9" s="8" t="str">
-        <x:v>Telefoonchat; eerdere context</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="45" customHeight="1">
+        <x:v>Hoofdchat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="55" customHeight="1">
       <x:c r="A10" s="8" t="str">
         <x:v>lasagne-classico</x:v>
       </x:c>
@@ -656,32 +692,32 @@
       <x:c r="C10" s="8" t="str">
         <x:v>Italiaans</x:v>
       </x:c>
-      <x:c r="D10" s="8" t="str">
-        <x:v>Concept – in review</x:v>
+      <x:c r="D10" s="15" t="str">
+        <x:v>Gepauzeerd</x:v>
       </x:c>
       <x:c r="E10" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Opnieuw te bepalen</x:v>
       </x:c>
       <x:c r="F10" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Opnieuw te bepalen</x:v>
       </x:c>
       <x:c r="G10" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Opnieuw te bepalen</x:v>
       </x:c>
       <x:c r="H10" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Nog vast te stellen</x:v>
       </x:c>
       <x:c r="I10" s="8" t="str">
-        <x:v>Nog verifiëren</x:v>
+        <x:v>Niet gepubliceerd bevestigd</x:v>
       </x:c>
       <x:c r="J10" s="8" t="str">
-        <x:v>Concept uit telefoonchat opnieuw nalopen; specifieke details nog niet bevestigd</x:v>
+        <x:v>Wacht op keuze van een ander basisrecept; geen inhoudelijke review plannen.</x:v>
       </x:c>
       <x:c r="K10" s="8" t="str">
         <x:v>Nog toe te wijzen</x:v>
       </x:c>
       <x:c r="L10" s="8" t="str">
-        <x:v>Telefoonchat; eerdere context</x:v>
+        <x:v>Hoofdchat</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -695,7 +731,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R264ca45502ee4315"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb7142d4c0dd40e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -735,7 +771,7 @@
         <x:v>Belangrijk</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>Het CSV-bestand is de centrale lijst; de individuele data/recepten/*.json-bestanden blijven de bron voor de website.</x:v>
+        <x:v>De Excel/CSV is het reviewoverzicht; de receptbestanden in data/recepten/*.json zijn leidend voor de website.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="47" customHeight="1">
@@ -775,7 +811,7 @@
         <x:v>Let op</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>Statussen van recepten uit de telefoonchat zijn gebaseerd op onze eerdere notities; de volledige conceptbestanden zijn hier niet opnieuw ingezien.</x:v>
+        <x:v>Status per 24 oktober 2026: 7 inhoudelijk afgeronde recepten, 1 historische variant geïntegreerd als weetje en 1 gepauzeerd. GitHub-publicatie niet overal geverifieerd.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="47" customHeight="1">
@@ -792,6 +828,68 @@
       </x:c>
       <x:c r="B11" s="8" t="str">
         <x:v>Na elke reviewsessie het overzicht opslaan en samen met de gewijzigde JSON naar GitHub committen.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="49" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>WORLD CUISINE — STATUS 24-10-2026</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="str">
+        <x:v>Aantal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" t="str">
+        <x:v>Inhoudelijk afgerond</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
+        <x:f>COUNTIF(Receptenoverzicht!D2:D10,"Inhoudelijk afgerond")</x:f>
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" t="str">
+        <x:v>Historisch weetje geïntegreerd</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:f>COUNTIF(Receptenoverzicht!D2:D10,"Geïntegreerd als weetje")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="25" customHeight="1">
+      <x:c r="A4" t="str">
+        <x:v>Gepauzeerd</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:f>COUNTIF(Receptenoverzicht!D2:D10,"Gepauzeerd")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" t="str">
+        <x:v>Totaal geregistreerd</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:f>SUM(B2:B4)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Publicatie op GitHub moet afzonderlijk worden gecontroleerd.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>